<commit_message>
Visites : type « Feuille de route » (revue budgétaire), reprise à l'import
Nouveau type de visite, avec compte rendu, qui ne compte pas dans le rythme
de visite. L'import lit les colonnes « Feuille de route » (OUI, OK, X, 1) et
crée une feuille de route à la date choisie pour les audits.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PHhMXCoZwUGUghubjdymnb
</commit_message>
<xml_diff>
--- a/tests/fichiers/suivi-visites-fictif.xlsx
+++ b/tests/fichiers/suivi-visites-fictif.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -602,6 +602,11 @@
           <t>Passage client mystère</t>
         </is>
       </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Feuille de route + prévi 2026</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="B12" t="inlineStr">
@@ -631,6 +636,11 @@
       <c r="H12" t="n">
         <v>0.5</v>
       </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>OUI</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="B13" t="inlineStr">
@@ -646,6 +656,11 @@
       <c r="F13" t="inlineStr">
         <is>
           <t>NON</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>x</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Import des visites : type et note à côté de chaque visite, sans commentaire
Une ligne par magasin ; chaque visite peut avoir une colonne « Type N »
(Visite terrain, Audit hygiène, Audit excellence, Feuille de route…) et une
colonne « Note N » : la note d'un audit est rangée à la date de la visite.
La colonne « Commentaire dernière visite » n'est plus reprise.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PHhMXCoZwUGUghubjdymnb
</commit_message>
<xml_diff>
--- a/tests/fichiers/suivi-visites-fictif.xlsx
+++ b/tests/fichiers/suivi-visites-fictif.xlsx
@@ -8,9 +8,10 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HUGO 2026" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INES 2026" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ZORRO 2026" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GLOBAL" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CAMILLE 2026" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INES 2026" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ZORRO 2026" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GLOBAL" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -675,13 +676,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Magasin </t>
+          <t>Magasin</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -691,18 +692,69 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>Type 1</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Note 1</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>Visite 2</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Type 2</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Note 2</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>V AND B NANTES TEST</t>
+          <t>Lyon Test</t>
         </is>
       </c>
       <c r="B2" s="1" t="n">
-        <v>46161</v>
+        <v>46083</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Audit hygiène</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="E2" s="1" t="n">
+        <v>46122</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Feuille de route</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Annecy Test</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="n">
+        <v>46054</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Visite terrain</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -739,16 +791,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Bordeaux Test</t>
+          <t>V AND B NANTES TEST</t>
         </is>
       </c>
       <c r="B2" s="1" t="n">
-        <v>46056</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>28 et 29/04/26</t>
-        </is>
+        <v>46161</v>
       </c>
     </row>
   </sheetData>
@@ -768,6 +815,52 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t xml:space="preserve">Magasin </t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Visite 1</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Visite 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Bordeaux Test</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="n">
+        <v>46056</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>28 et 29/04/26</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
           <t>MAGASIN</t>
         </is>
       </c>

</xml_diff>